<commit_message>
Update model outputs 2026-09-13 09:41:09
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,49 +44,13 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kennedy Community Centre</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unley Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mineral Resources Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
   </si>
   <si>
     <t xml:space="preserve">Casey Fields</t>
@@ -461,7 +425,7 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="17.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
@@ -469,7 +433,7 @@
     <col min="7" max="7" width="24.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="26.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="15.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="24.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="17.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,7 +470,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -521,16 +485,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>6.3</v>
+        <v>-30.3</v>
       </c>
       <c r="G2" t="n">
-        <v>7.1</v>
+        <v>-10.2</v>
       </c>
       <c r="H2" t="n">
-        <v>9.6</v>
+        <v>-34.1</v>
       </c>
       <c r="I2" t="n">
-        <v>76.1</v>
+        <v>95.1</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -538,7 +502,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -553,16 +517,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>-11.1</v>
+        <v>7.2</v>
       </c>
       <c r="G3" t="n">
-        <v>6.1</v>
+        <v>3.1</v>
       </c>
       <c r="H3" t="n">
-        <v>-11.7</v>
+        <v>17</v>
       </c>
       <c r="I3" t="n">
-        <v>78.7</v>
+        <v>77.2</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -570,7 +534,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -585,16 +549,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-8.2</v>
+        <v>-30.3</v>
       </c>
       <c r="G4" t="n">
-        <v>-5.9</v>
+        <v>-12.5</v>
       </c>
       <c r="H4" t="n">
-        <v>-9.2</v>
+        <v>-34.2</v>
       </c>
       <c r="I4" t="n">
-        <v>85.5</v>
+        <v>87.8</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -602,7 +566,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46277</v>
+        <v>46278</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -617,16 +581,16 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>20.1</v>
+        <v>-48.3</v>
       </c>
       <c r="G5" t="n">
-        <v>11.4</v>
+        <v>-19.7</v>
       </c>
       <c r="H5" t="n">
-        <v>16.9</v>
+        <v>-47.3</v>
       </c>
       <c r="I5" t="n">
-        <v>81.2</v>
+        <v>89.4</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -649,147 +613,19 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>-30.3</v>
+        <v>-16.2</v>
       </c>
       <c r="G6" t="n">
-        <v>-10.2</v>
+        <v>-9.5</v>
       </c>
       <c r="H6" t="n">
-        <v>-34.1</v>
+        <v>-14.2</v>
       </c>
       <c r="I6" t="n">
-        <v>95.1</v>
+        <v>73.3</v>
       </c>
       <c r="J6" t="s">
         <v>25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="G7" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>17</v>
-      </c>
-      <c r="I7" t="n">
-        <v>77.2</v>
-      </c>
-      <c r="J7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-30.3</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-12.5</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-34.2</v>
-      </c>
-      <c r="I8" t="n">
-        <v>87.8</v>
-      </c>
-      <c r="J8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-48.3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>-19.7</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-47.3</v>
-      </c>
-      <c r="I9" t="n">
-        <v>89.4</v>
-      </c>
-      <c r="J9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46278</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-16.2</v>
-      </c>
-      <c r="G10" t="n">
-        <v>-9.5</v>
-      </c>
-      <c r="H10" t="n">
-        <v>-14.2</v>
-      </c>
-      <c r="I10" t="n">
-        <v>73.3</v>
-      </c>
-      <c r="J10" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-09-19 12:08:54
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,22 +44,13 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cazalys Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
   </si>
   <si>
     <t xml:space="preserve">Victoria Park</t>
@@ -506,7 +497,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46283</v>
+        <v>46284</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -521,16 +512,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>47.3</v>
+        <v>25.8</v>
       </c>
       <c r="G2" t="n">
-        <v>27.3</v>
+        <v>8</v>
       </c>
       <c r="H2" t="n">
-        <v>51.9</v>
+        <v>23.9</v>
       </c>
       <c r="I2" t="n">
-        <v>82.3</v>
+        <v>78.9</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -553,16 +544,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>25.8</v>
+        <v>-26</v>
       </c>
       <c r="G3" t="n">
-        <v>8</v>
+        <v>-6.1</v>
       </c>
       <c r="H3" t="n">
-        <v>23.9</v>
+        <v>-30</v>
       </c>
       <c r="I3" t="n">
-        <v>78.9</v>
+        <v>90.3</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -585,16 +576,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-26</v>
+        <v>8.4</v>
       </c>
       <c r="G4" t="n">
-        <v>-6.1</v>
+        <v>-4.7</v>
       </c>
       <c r="H4" t="n">
-        <v>-30</v>
+        <v>12.9</v>
       </c>
       <c r="I4" t="n">
-        <v>90.3</v>
+        <v>93</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -617,16 +608,16 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>8.4</v>
+        <v>-0.9</v>
       </c>
       <c r="G5" t="n">
-        <v>-4.7</v>
+        <v>3.8</v>
       </c>
       <c r="H5" t="n">
-        <v>12.9</v>
+        <v>-1.7</v>
       </c>
       <c r="I5" t="n">
-        <v>93</v>
+        <v>73.7</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -634,7 +625,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -649,16 +640,16 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.9</v>
+        <v>0.5</v>
       </c>
       <c r="G6" t="n">
-        <v>3.8</v>
+        <v>2.4</v>
       </c>
       <c r="H6" t="n">
-        <v>-1.7</v>
+        <v>-6.5</v>
       </c>
       <c r="I6" t="n">
-        <v>73.7</v>
+        <v>85.1</v>
       </c>
       <c r="J6" t="s">
         <v>25</v>
@@ -681,16 +672,16 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>0.5</v>
+        <v>1.7</v>
       </c>
       <c r="G7" t="n">
-        <v>2.4</v>
+        <v>-9.2</v>
       </c>
       <c r="H7" t="n">
-        <v>-6.5</v>
+        <v>-1.5</v>
       </c>
       <c r="I7" t="n">
-        <v>85.1</v>
+        <v>80.3</v>
       </c>
       <c r="J7" t="s">
         <v>28</v>
@@ -713,16 +704,16 @@
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>1.7</v>
+        <v>6.3</v>
       </c>
       <c r="G8" t="n">
-        <v>-9.2</v>
+        <v>1.3</v>
       </c>
       <c r="H8" t="n">
-        <v>-1.5</v>
+        <v>6</v>
       </c>
       <c r="I8" t="n">
-        <v>80.3</v>
+        <v>75.8</v>
       </c>
       <c r="J8" t="s">
         <v>31</v>
@@ -745,51 +736,19 @@
         <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>6.3</v>
+        <v>-7.9</v>
       </c>
       <c r="G9" t="n">
-        <v>1.3</v>
+        <v>-9.7</v>
       </c>
       <c r="H9" t="n">
-        <v>6</v>
+        <v>-8.8</v>
       </c>
       <c r="I9" t="n">
-        <v>75.8</v>
+        <v>85.6</v>
       </c>
       <c r="J9" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46285</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-7.9</v>
-      </c>
-      <c r="G10" t="n">
-        <v>-9.7</v>
-      </c>
-      <c r="H10" t="n">
-        <v>-8.8</v>
-      </c>
-      <c r="I10" t="n">
-        <v>85.6</v>
-      </c>
-      <c r="J10" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-09-20 05:30:12
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,49 +44,13 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Victoria Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Casey Fields</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alberton Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cockburn ARC Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
   </si>
   <si>
     <t xml:space="preserve">Corroboree Group Oval Manuka</t>
@@ -497,7 +461,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -512,16 +476,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>25.8</v>
+        <v>0.5</v>
       </c>
       <c r="G2" t="n">
-        <v>8</v>
+        <v>2.4</v>
       </c>
       <c r="H2" t="n">
-        <v>23.9</v>
+        <v>-6.5</v>
       </c>
       <c r="I2" t="n">
-        <v>78.9</v>
+        <v>85.1</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -529,7 +493,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -544,16 +508,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>-26</v>
+        <v>1.7</v>
       </c>
       <c r="G3" t="n">
-        <v>-6.1</v>
+        <v>-9.2</v>
       </c>
       <c r="H3" t="n">
-        <v>-30</v>
+        <v>-1.5</v>
       </c>
       <c r="I3" t="n">
-        <v>90.3</v>
+        <v>80.3</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -561,7 +525,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -576,16 +540,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>8.4</v>
+        <v>6.3</v>
       </c>
       <c r="G4" t="n">
-        <v>-4.7</v>
+        <v>1.3</v>
       </c>
       <c r="H4" t="n">
-        <v>12.9</v>
+        <v>6</v>
       </c>
       <c r="I4" t="n">
-        <v>93</v>
+        <v>75.8</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -593,7 +557,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46284</v>
+        <v>46285</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -608,147 +572,19 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.9</v>
+        <v>-7.9</v>
       </c>
       <c r="G5" t="n">
-        <v>3.8</v>
+        <v>-9.7</v>
       </c>
       <c r="H5" t="n">
-        <v>-1.7</v>
+        <v>-8.8</v>
       </c>
       <c r="I5" t="n">
-        <v>73.7</v>
+        <v>85.6</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46285</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-6.5</v>
-      </c>
-      <c r="I6" t="n">
-        <v>85.1</v>
-      </c>
-      <c r="J6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46285</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-9.2</v>
-      </c>
-      <c r="H7" t="n">
-        <v>-1.5</v>
-      </c>
-      <c r="I7" t="n">
-        <v>80.3</v>
-      </c>
-      <c r="J7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46285</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="H8" t="n">
-        <v>6</v>
-      </c>
-      <c r="I8" t="n">
-        <v>75.8</v>
-      </c>
-      <c r="J8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46285</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-7.9</v>
-      </c>
-      <c r="G9" t="n">
-        <v>-9.7</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-8.8</v>
-      </c>
-      <c r="I9" t="n">
-        <v>85.6</v>
-      </c>
-      <c r="J9" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NBL projections 2026-09-25 11:47:17
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -42,18 +42,6 @@
   </si>
   <si>
     <t xml:space="preserve">Venue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Provisional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GMHBA Stadium</t>
   </si>
   <si>
     <t xml:space="preserve">essendon</t>
@@ -506,7 +494,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -521,16 +509,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>-19.9</v>
+        <v>-4</v>
       </c>
       <c r="G2" t="n">
-        <v>-2.2</v>
+        <v>5.1</v>
       </c>
       <c r="H2" t="n">
-        <v>-23.5</v>
+        <v>-9.2</v>
       </c>
       <c r="I2" t="n">
-        <v>83</v>
+        <v>73.9</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -547,25 +535,25 @@
         <v>15</v>
       </c>
       <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-17.7</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-3.9</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-19.5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="J3" t="s">
         <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-4</v>
-      </c>
-      <c r="G3" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-9.2</v>
-      </c>
-      <c r="I3" t="n">
-        <v>73.9</v>
-      </c>
-      <c r="J3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -573,31 +561,31 @@
         <v>46290</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-26.3</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-13.4</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-34.7</v>
+      </c>
+      <c r="I4" t="n">
+        <v>85.1</v>
+      </c>
+      <c r="J4" t="s">
         <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-17.7</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-3.9</v>
-      </c>
-      <c r="H4" t="n">
-        <v>-19.5</v>
-      </c>
-      <c r="I4" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="J4" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="5">
@@ -605,63 +593,63 @@
         <v>46290</v>
       </c>
       <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
         <v>21</v>
       </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>-26.3</v>
+        <v>7.5</v>
       </c>
       <c r="G5" t="n">
-        <v>-13.4</v>
+        <v>13.3</v>
       </c>
       <c r="H5" t="n">
-        <v>-34.7</v>
+        <v>7.2</v>
       </c>
       <c r="I5" t="n">
-        <v>85.1</v>
+        <v>87.8</v>
       </c>
       <c r="J5" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-6.2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>-7.9</v>
+      </c>
+      <c r="I6" t="n">
+        <v>81.5</v>
+      </c>
+      <c r="J6" t="s">
         <v>24</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-      <c r="D6" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>13.3</v>
-      </c>
-      <c r="H6" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="I6" t="n">
-        <v>87.8</v>
-      </c>
-      <c r="J6" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="7">
@@ -669,31 +657,31 @@
         <v>46292</v>
       </c>
       <c r="B7" t="s">
+        <v>25</v>
+      </c>
+      <c r="C7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-11.1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-6.9</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-12</v>
+      </c>
+      <c r="I7" t="n">
+        <v>78.3</v>
+      </c>
+      <c r="J7" t="s">
         <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" t="n">
-        <v>-6.9</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-6.2</v>
-      </c>
-      <c r="H7" t="n">
-        <v>-7.9</v>
-      </c>
-      <c r="I7" t="n">
-        <v>81.5</v>
-      </c>
-      <c r="J7" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="8">
@@ -701,31 +689,31 @@
         <v>46292</v>
       </c>
       <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
         <v>29</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="G8" t="n">
+        <v>9</v>
+      </c>
+      <c r="H8" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>86.1</v>
+      </c>
+      <c r="J8" t="s">
         <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-11.1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-6.9</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-12</v>
-      </c>
-      <c r="I8" t="n">
-        <v>78.3</v>
-      </c>
-      <c r="J8" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -733,63 +721,31 @@
         <v>46292</v>
       </c>
       <c r="B9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" t="s">
         <v>32</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-15.1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-11.9</v>
+      </c>
+      <c r="I9" t="n">
+        <v>81.8</v>
+      </c>
+      <c r="J9" t="s">
         <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>9</v>
-      </c>
-      <c r="H9" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="I9" t="n">
-        <v>86.1</v>
-      </c>
-      <c r="J9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-15.1</v>
-      </c>
-      <c r="G10" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="H10" t="n">
-        <v>-11.9</v>
-      </c>
-      <c r="I10" t="n">
-        <v>81.8</v>
-      </c>
-      <c r="J10" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NBL projections 2026-09-26 08:09:47
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,76 +44,52 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
   </si>
   <si>
-    <t xml:space="preserve">Windy Hill</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mission Whitten Oval</t>
+    <t xml:space="preserve">Victoria Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unley Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Henson Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People First Stadium</t>
   </si>
   <si>
     <t xml:space="preserve">carlton</t>
   </si>
   <si>
-    <t xml:space="preserve">richmond</t>
+    <t xml:space="preserve">hawthorn</t>
   </si>
   <si>
     <t xml:space="preserve">IKON Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Victoria Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unley Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Henson Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
   </si>
 </sst>
 </file>
@@ -449,7 +425,7 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
@@ -494,7 +470,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -509,16 +485,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>-4</v>
+        <v>-6.9</v>
       </c>
       <c r="G2" t="n">
-        <v>5.1</v>
+        <v>-6.2</v>
       </c>
       <c r="H2" t="n">
-        <v>-9.2</v>
+        <v>-7.9</v>
       </c>
       <c r="I2" t="n">
-        <v>73.9</v>
+        <v>81.5</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -526,7 +502,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -541,16 +517,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>-17.7</v>
+        <v>-11.1</v>
       </c>
       <c r="G3" t="n">
-        <v>-3.9</v>
+        <v>-6.9</v>
       </c>
       <c r="H3" t="n">
-        <v>-19.5</v>
+        <v>-12</v>
       </c>
       <c r="I3" t="n">
-        <v>87.5</v>
+        <v>78.3</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -558,7 +534,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -573,16 +549,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-26.3</v>
+        <v>10.3</v>
       </c>
       <c r="G4" t="n">
-        <v>-13.4</v>
+        <v>9</v>
       </c>
       <c r="H4" t="n">
-        <v>-34.7</v>
+        <v>10.3</v>
       </c>
       <c r="I4" t="n">
-        <v>85.1</v>
+        <v>86.1</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -590,7 +566,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -605,30 +581,30 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>7.5</v>
+        <v>-15.1</v>
       </c>
       <c r="G5" t="n">
-        <v>13.3</v>
+        <v>8.4</v>
       </c>
       <c r="H5" t="n">
-        <v>7.2</v>
+        <v>-11.9</v>
       </c>
       <c r="I5" t="n">
-        <v>87.8</v>
+        <v>81.8</v>
       </c>
       <c r="J5" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -637,115 +613,19 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>-6.9</v>
+        <v>-13.2</v>
       </c>
       <c r="G6" t="n">
-        <v>-6.2</v>
+        <v>-7.4</v>
       </c>
       <c r="H6" t="n">
-        <v>-7.9</v>
+        <v>-17.8</v>
       </c>
       <c r="I6" t="n">
-        <v>81.5</v>
+        <v>84.5</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B7" t="s">
         <v>25</v>
-      </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="n">
-        <v>-11.1</v>
-      </c>
-      <c r="G7" t="n">
-        <v>-6.9</v>
-      </c>
-      <c r="H7" t="n">
-        <v>-12</v>
-      </c>
-      <c r="I7" t="n">
-        <v>78.3</v>
-      </c>
-      <c r="J7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B8" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="G8" t="n">
-        <v>9</v>
-      </c>
-      <c r="H8" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="I8" t="n">
-        <v>86.1</v>
-      </c>
-      <c r="J8" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-15.1</v>
-      </c>
-      <c r="G9" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-11.9</v>
-      </c>
-      <c r="I9" t="n">
-        <v>81.8</v>
-      </c>
-      <c r="J9" t="s">
-        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NBL projections 2026-09-29 20:17:40
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,49 +44,13 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Victoria Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unley Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Henson Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
   </si>
   <si>
     <t xml:space="preserve">IKON Park</t>
@@ -425,15 +389,15 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="9.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="24.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="26.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="15.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="20.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="9.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -470,7 +434,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46292</v>
+        <v>46296</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -485,147 +449,19 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>-6.9</v>
+        <v>-13.2</v>
       </c>
       <c r="G2" t="n">
-        <v>-6.2</v>
+        <v>-7.4</v>
       </c>
       <c r="H2" t="n">
-        <v>-7.9</v>
+        <v>-17.8</v>
       </c>
       <c r="I2" t="n">
-        <v>81.5</v>
+        <v>84.5</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-11.1</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-6.9</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-12</v>
-      </c>
-      <c r="I3" t="n">
-        <v>78.3</v>
-      </c>
-      <c r="J3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="G4" t="n">
-        <v>9</v>
-      </c>
-      <c r="H4" t="n">
-        <v>10.3</v>
-      </c>
-      <c r="I4" t="n">
-        <v>86.1</v>
-      </c>
-      <c r="J4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46292</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-15.1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="H5" t="n">
-        <v>-11.9</v>
-      </c>
-      <c r="I5" t="n">
-        <v>81.8</v>
-      </c>
-      <c r="J5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46296</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-13.2</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-7.4</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-17.8</v>
-      </c>
-      <c r="I6" t="n">
-        <v>84.5</v>
-      </c>
-      <c r="J6" t="s">
-        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refresh NRL, NRLW and AFLW model outputs 2026-10-02
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,16 +44,79 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
   </si>
   <si>
     <t xml:space="preserve">IKON Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Henson Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mars Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brighton Homes Arena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alberton Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arden Street Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Victoria Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">west coast eagles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sullivan Logistics Stadium</t>
   </si>
 </sst>
 </file>
@@ -389,15 +452,15 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="9.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="9.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="15.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="24.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="26.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="15.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="9.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="26.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -434,7 +497,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46296</v>
+        <v>46297</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -449,19 +512,243 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>-13.2</v>
+        <v>31.2</v>
       </c>
       <c r="G2" t="n">
-        <v>-7.4</v>
+        <v>8.5</v>
       </c>
       <c r="H2" t="n">
-        <v>-17.8</v>
+        <v>38.2</v>
       </c>
       <c r="I2" t="n">
-        <v>84.5</v>
+        <v>83.9</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="I3" t="n">
+        <v>82.5</v>
+      </c>
+      <c r="J3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-29.5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-10.2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-29.7</v>
+      </c>
+      <c r="I4" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="J4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-13.9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-26.6</v>
+      </c>
+      <c r="H5" t="n">
+        <v>-16.4</v>
+      </c>
+      <c r="I5" t="n">
+        <v>87.4</v>
+      </c>
+      <c r="J5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="H6" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="I6" t="n">
+        <v>92.3</v>
+      </c>
+      <c r="J6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="n">
+        <v>-44</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-26.5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>-51.4</v>
+      </c>
+      <c r="I7" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="J7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>31</v>
+      </c>
+      <c r="G8" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="H8" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="I8" t="n">
+        <v>79.9</v>
+      </c>
+      <c r="J8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H9" t="n">
+        <v>9</v>
+      </c>
+      <c r="I9" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="J9" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NBL projections 2026-10-03 15:11:38
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,22 +44,13 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IKON Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
   </si>
   <si>
     <t xml:space="preserve">Henson Park</t>
@@ -497,7 +488,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46297</v>
+        <v>46298</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -512,16 +503,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>31.2</v>
+        <v>11.3</v>
       </c>
       <c r="G2" t="n">
-        <v>8.5</v>
+        <v>1.5</v>
       </c>
       <c r="H2" t="n">
-        <v>38.2</v>
+        <v>17.3</v>
       </c>
       <c r="I2" t="n">
-        <v>83.9</v>
+        <v>82.5</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -544,16 +535,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>11.3</v>
+        <v>-29.5</v>
       </c>
       <c r="G3" t="n">
-        <v>1.5</v>
+        <v>-10.2</v>
       </c>
       <c r="H3" t="n">
-        <v>17.3</v>
+        <v>-29.7</v>
       </c>
       <c r="I3" t="n">
-        <v>82.5</v>
+        <v>75.5</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -576,16 +567,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-29.5</v>
+        <v>-13.9</v>
       </c>
       <c r="G4" t="n">
-        <v>-10.2</v>
+        <v>-26.6</v>
       </c>
       <c r="H4" t="n">
-        <v>-29.7</v>
+        <v>-16.4</v>
       </c>
       <c r="I4" t="n">
-        <v>75.5</v>
+        <v>87.4</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -608,16 +599,16 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>-13.9</v>
+        <v>16.1</v>
       </c>
       <c r="G5" t="n">
-        <v>-26.6</v>
+        <v>0.9</v>
       </c>
       <c r="H5" t="n">
-        <v>-16.4</v>
+        <v>19.1</v>
       </c>
       <c r="I5" t="n">
-        <v>87.4</v>
+        <v>92.3</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -625,7 +616,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -640,16 +631,16 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>16.1</v>
+        <v>-44</v>
       </c>
       <c r="G6" t="n">
-        <v>0.9</v>
+        <v>-26.5</v>
       </c>
       <c r="H6" t="n">
-        <v>19.1</v>
+        <v>-51.4</v>
       </c>
       <c r="I6" t="n">
-        <v>92.3</v>
+        <v>85.5</v>
       </c>
       <c r="J6" t="s">
         <v>25</v>
@@ -672,16 +663,16 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>-44</v>
+        <v>31</v>
       </c>
       <c r="G7" t="n">
-        <v>-26.5</v>
+        <v>19.7</v>
       </c>
       <c r="H7" t="n">
-        <v>-51.4</v>
+        <v>31.6</v>
       </c>
       <c r="I7" t="n">
-        <v>85.5</v>
+        <v>79.9</v>
       </c>
       <c r="J7" t="s">
         <v>28</v>
@@ -704,51 +695,19 @@
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>31</v>
+        <v>11.3</v>
       </c>
       <c r="G8" t="n">
-        <v>19.7</v>
+        <v>0.8</v>
       </c>
       <c r="H8" t="n">
-        <v>31.6</v>
+        <v>9</v>
       </c>
       <c r="I8" t="n">
-        <v>79.9</v>
+        <v>74.2</v>
       </c>
       <c r="J8" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46299</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H9" t="n">
-        <v>9</v>
-      </c>
-      <c r="I9" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="J9" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore full Greyhound form and pricing display
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,49 +44,13 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Henson Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mars Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brighton Homes Arena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alberton Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
   </si>
   <si>
     <t xml:space="preserve">Arden Street Oval</t>
@@ -443,8 +407,8 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="15.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="17.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
@@ -488,7 +452,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -503,16 +467,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>11.3</v>
+        <v>-44</v>
       </c>
       <c r="G2" t="n">
-        <v>1.5</v>
+        <v>-26.5</v>
       </c>
       <c r="H2" t="n">
-        <v>17.3</v>
+        <v>-51.4</v>
       </c>
       <c r="I2" t="n">
-        <v>82.5</v>
+        <v>85.5</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -520,7 +484,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -535,16 +499,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>-29.5</v>
+        <v>31</v>
       </c>
       <c r="G3" t="n">
-        <v>-10.2</v>
+        <v>19.7</v>
       </c>
       <c r="H3" t="n">
-        <v>-29.7</v>
+        <v>31.6</v>
       </c>
       <c r="I3" t="n">
-        <v>75.5</v>
+        <v>79.9</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -552,7 +516,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -567,147 +531,19 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-13.9</v>
+        <v>11.3</v>
       </c>
       <c r="G4" t="n">
-        <v>-26.6</v>
+        <v>0.8</v>
       </c>
       <c r="H4" t="n">
-        <v>-16.4</v>
+        <v>9</v>
       </c>
       <c r="I4" t="n">
-        <v>87.4</v>
+        <v>74.2</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46298</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="n">
-        <v>16.1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="H5" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="I5" t="n">
-        <v>92.3</v>
-      </c>
-      <c r="J5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46299</v>
-      </c>
-      <c r="B6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-44</v>
-      </c>
-      <c r="G6" t="n">
-        <v>-26.5</v>
-      </c>
-      <c r="H6" t="n">
-        <v>-51.4</v>
-      </c>
-      <c r="I6" t="n">
-        <v>85.5</v>
-      </c>
-      <c r="J6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46299</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="n">
-        <v>31</v>
-      </c>
-      <c r="G7" t="n">
-        <v>19.7</v>
-      </c>
-      <c r="H7" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="I7" t="n">
-        <v>79.9</v>
-      </c>
-      <c r="J7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46299</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="H8" t="n">
-        <v>9</v>
-      </c>
-      <c r="I8" t="n">
-        <v>74.2</v>
-      </c>
-      <c r="J8" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>